<commit_message>
Clarify language recall presentation
</commit_message>
<xml_diff>
--- a/public/downloads/holorecall-blank-v5.xlsx
+++ b/public/downloads/holorecall-blank-v5.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="65">
   <si>
     <t>key</t>
   </si>
@@ -26,7 +26,7 @@
     <t>format_version</t>
   </si>
   <si>
-    <t>5</t>
+    <t>9</t>
   </si>
   <si>
     <t>content_only</t>
@@ -56,6 +56,12 @@
     <t>anki_source</t>
   </si>
   <si>
+    <t>cover_media</t>
+  </si>
+  <si>
+    <t>study_art_policy</t>
+  </si>
+  <si>
     <t>card_id</t>
   </si>
   <si>
@@ -104,6 +110,27 @@
     <t>sibling_group_id</t>
   </si>
   <si>
+    <t>art</t>
+  </si>
+  <si>
+    <t>choices</t>
+  </si>
+  <si>
+    <t>answer_label</t>
+  </si>
+  <si>
+    <t>details</t>
+  </si>
+  <si>
+    <t>secondary</t>
+  </si>
+  <si>
+    <t>interpretation</t>
+  </si>
+  <si>
+    <t>presentation</t>
+  </si>
+  <si>
     <t>name</t>
   </si>
   <si>
@@ -165,6 +192,9 @@
   </si>
   <si>
     <t>texture</t>
+  </si>
+  <si>
+    <t>design_schema</t>
   </si>
   <si>
     <t>asset_id</t>
@@ -610,13 +640,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="7" width="18" customWidth="1"/>
+    <col min="1" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -638,9 +668,15 @@
       <c r="G1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -648,76 +684,97 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="20" width="18" customWidth="1"/>
+    <col min="1" max="27" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="U1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T1"/>
+  <autoFilter ref="A1:AA1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -725,84 +782,87 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="12" width="18" customWidth="1"/>
     <col min="13" max="14" width="21" customWidth="1"/>
-    <col min="15" max="22" width="18" customWidth="1"/>
+    <col min="15" max="23" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>49</v>
+        <v>58</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V1"/>
+  <autoFilter ref="A1:W1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -818,31 +878,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>